<commit_message>
Two of his workbooks that put a column on a page of its own on A4 now fit the page's width: F/PUR/03's approved suppliers and F/PRD/24's blade record (REQUIREMENTS section 119)
The A4 print of every workbook that downloads as his file (Excel's own PDF, with Excel's "scale content for A4 or 8.5 x 11"
off in the check's own Excel so the sheet prints on its own A4) found two whose printed columns are wider than A4 between his
margins at his own scale, on his own A4 setting: F/PUR/03 (60 %, 947 pt of columns on 842 pt) printed its last two columns
and the format number's end on a second page, F/PRD/24 (67 %, 578 pt on 559 pt) its last column. scripts/originals/convert.py
now has Excel fit such a sheet to the page's width (one page across, the length left to run), for every workbook, A4 or not;
the two are made again from his originals and print on one page each. The other 34 workbooks fit across at his scale.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/originals/prd-slitting-blade.xlsx
+++ b/frontend/public/originals/prd-slitting-blade.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parth\Desktop\dcrs-orig-wt\frontend\public\originals\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{33FD2FBB-546A-49BB-B3CB-26E337103DD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8831CBD5-9341-44D1-ACE6-6127757C3EE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -728,6 +728,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:J34"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1765,7 +1768,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.39" bottom="0.25" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="67" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="64" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <colBreaks count="1" manualBreakCount="1">
     <brk id="10" max="1048575" man="1"/>
   </colBreaks>

</xml_diff>